<commit_message>
Added models on buffer 40
</commit_message>
<xml_diff>
--- a/learning/gesture.xlsx
+++ b/learning/gesture.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\user\project\slovo\learning\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD2CE0CB-0B44-487C-ABB8-81150C32969B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4957E9F-A8B5-4F7F-A99F-D32546FBEC8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{31CF1E62-7D6D-4D80-B7A8-01836A8AAD2A}"/>
+    <workbookView xWindow="3510" yWindow="3510" windowWidth="21600" windowHeight="11280" xr2:uid="{31CF1E62-7D6D-4D80-B7A8-01836A8AAD2A}"/>
   </bookViews>
   <sheets>
     <sheet name="Лист1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="28">
   <si>
     <t>0.5</t>
   </si>
@@ -111,6 +111,18 @@
   </si>
   <si>
     <t>gesture-wbw-60-3</t>
+  </si>
+  <si>
+    <t>gesture-bw-60-1</t>
+  </si>
+  <si>
+    <t>avg+max+min+std pool</t>
+  </si>
+  <si>
+    <t>512 0.5</t>
+  </si>
+  <si>
+    <t>256 0.4</t>
   </si>
 </sst>
 </file>
@@ -149,12 +161,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -170,7 +188,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -180,12 +198,19 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="2" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="9" fontId="0" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="10" fontId="0" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -525,17 +550,17 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
-    <col min="2" max="2" width="13.28515625" customWidth="1"/>
+    <col min="2" max="2" width="23" customWidth="1"/>
     <col min="3" max="3" width="17.7109375" customWidth="1"/>
     <col min="4" max="4" width="10.42578125" customWidth="1"/>
     <col min="5" max="5" width="9.5703125" customWidth="1"/>
     <col min="9" max="9" width="29" customWidth="1"/>
     <col min="10" max="10" width="12.7109375" customWidth="1"/>
-    <col min="12" max="12" width="9.140625" style="6"/>
+    <col min="12" max="12" width="9.140625" style="5"/>
     <col min="13" max="13" width="9.140625" style="2"/>
-    <col min="14" max="14" width="9.140625" style="6"/>
-    <col min="16" max="16" width="9.140625" style="6"/>
-    <col min="18" max="18" width="9.140625" style="6"/>
+    <col min="14" max="14" width="9.140625" style="5"/>
+    <col min="16" max="16" width="9.140625" style="5"/>
+    <col min="18" max="18" width="9.140625" style="5"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:25" x14ac:dyDescent="0.25">
@@ -548,40 +573,40 @@
       <c r="I1" t="s">
         <v>4</v>
       </c>
-      <c r="K1" s="5" t="s">
+      <c r="K1" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="L1" s="5"/>
-      <c r="M1" s="5"/>
-      <c r="N1" s="5"/>
-      <c r="O1" s="5"/>
-      <c r="P1" s="5"/>
-      <c r="Q1" s="5"/>
-      <c r="R1" s="5"/>
+      <c r="L1" s="8"/>
+      <c r="M1" s="8"/>
+      <c r="N1" s="8"/>
+      <c r="O1" s="8"/>
+      <c r="P1" s="8"/>
+      <c r="Q1" s="8"/>
+      <c r="R1" s="8"/>
     </row>
     <row r="2" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="K2" s="5" t="s">
+      <c r="K2" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="L2" s="5"/>
-      <c r="M2" s="5" t="s">
+      <c r="L2" s="8"/>
+      <c r="M2" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="N2" s="5"/>
-      <c r="O2" s="5" t="s">
+      <c r="N2" s="8"/>
+      <c r="O2" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="P2" s="5"/>
-      <c r="Q2" s="5" t="s">
+      <c r="P2" s="8"/>
+      <c r="Q2" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="R2" s="5"/>
-      <c r="V2" s="5" t="s">
+      <c r="R2" s="8"/>
+      <c r="V2" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="W2" s="5"/>
-      <c r="X2" s="5"/>
-      <c r="Y2" s="5"/>
+      <c r="W2" s="8"/>
+      <c r="X2" s="8"/>
+      <c r="Y2" s="8"/>
     </row>
     <row r="3" spans="1:25" x14ac:dyDescent="0.25">
       <c r="J3" t="s">
@@ -590,28 +615,28 @@
       <c r="K3" t="s">
         <v>5</v>
       </c>
-      <c r="L3" s="6" t="s">
+      <c r="L3" s="5" t="s">
         <v>6</v>
       </c>
       <c r="M3" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="N3" s="6" t="s">
+      <c r="N3" s="5" t="s">
         <v>6</v>
       </c>
       <c r="O3" t="s">
         <v>5</v>
       </c>
-      <c r="P3" s="6" t="s">
+      <c r="P3" s="5" t="s">
         <v>6</v>
       </c>
       <c r="Q3" t="s">
         <v>5</v>
       </c>
-      <c r="R3" s="6" t="s">
+      <c r="R3" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="T3" s="6" t="s">
+      <c r="T3" s="5" t="s">
         <v>17</v>
       </c>
       <c r="V3" t="s">
@@ -627,68 +652,68 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
+    <row r="4" spans="1:25" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="E4" t="s">
+      <c r="E4" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="G4">
+      <c r="G4" s="10">
         <v>768</v>
       </c>
-      <c r="I4" t="s">
+      <c r="I4" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="J4">
+      <c r="J4" s="10">
         <v>0.98</v>
       </c>
-      <c r="K4" s="8">
+      <c r="K4" s="11">
         <v>0.68479571332886802</v>
       </c>
-      <c r="L4" s="6">
+      <c r="L4" s="12">
         <v>0</v>
       </c>
-      <c r="M4" s="8">
-        <v>8.1749049429657699E-3</v>
-      </c>
-      <c r="N4" s="6">
+      <c r="M4" s="11">
+        <v>0.81749049429657705</v>
+      </c>
+      <c r="N4" s="12">
         <v>0.26</v>
       </c>
-      <c r="O4" s="8">
+      <c r="O4" s="11">
         <v>0.90199081163859096</v>
       </c>
-      <c r="P4" s="6">
+      <c r="P4" s="12">
         <v>0.48</v>
       </c>
-      <c r="Q4" s="8">
+      <c r="Q4" s="11">
         <v>0.95996592844974404</v>
       </c>
-      <c r="R4" s="6">
+      <c r="R4" s="12">
         <v>0.69</v>
       </c>
-      <c r="T4" s="8">
+      <c r="T4" s="11">
         <v>0.86965840589417198</v>
       </c>
-      <c r="V4" s="2">
+      <c r="V4" s="13">
         <v>0.93774319066147804</v>
       </c>
-      <c r="W4" s="2">
+      <c r="W4" s="13">
         <v>0.78728923476005097</v>
       </c>
-      <c r="X4" s="2">
+      <c r="X4" s="13">
         <v>0.495460440985732</v>
       </c>
-      <c r="Y4" s="2">
+      <c r="Y4" s="13">
         <v>0.25162127107652399</v>
       </c>
     </row>
@@ -717,31 +742,31 @@
       <c r="J5" s="4">
         <v>0.95</v>
       </c>
-      <c r="K5" s="8">
+      <c r="K5" s="7">
         <v>0.68479571332886802</v>
       </c>
-      <c r="L5" s="7">
+      <c r="L5" s="6">
         <v>0</v>
       </c>
-      <c r="M5" s="8">
-        <v>8.1749049429657699E-3</v>
-      </c>
-      <c r="N5" s="7">
+      <c r="M5" s="7">
+        <v>0.81749049429657705</v>
+      </c>
+      <c r="N5" s="6">
         <v>0.26</v>
       </c>
-      <c r="O5" s="8">
+      <c r="O5" s="7">
         <v>0.90199081163859096</v>
       </c>
-      <c r="P5" s="7">
+      <c r="P5" s="6">
         <v>0.47</v>
       </c>
-      <c r="Q5" s="8">
+      <c r="Q5" s="7">
         <v>0.95996592844974404</v>
       </c>
-      <c r="R5" s="7">
+      <c r="R5" s="6">
         <v>0.69</v>
       </c>
-      <c r="T5" s="8">
+      <c r="T5" s="7">
         <v>0.86483590087073003</v>
       </c>
       <c r="V5" s="2">
@@ -776,31 +801,31 @@
       <c r="J6">
         <v>0.97</v>
       </c>
-      <c r="K6" s="8">
+      <c r="K6" s="7">
         <v>0.65612860013395802</v>
       </c>
-      <c r="L6" s="6">
+      <c r="L6" s="5">
         <v>0</v>
       </c>
-      <c r="M6" s="8">
+      <c r="M6" s="7">
         <v>0.79122115925717496</v>
       </c>
-      <c r="N6" s="6">
+      <c r="N6" s="5">
         <v>0.28999999999999998</v>
       </c>
-      <c r="O6" s="8">
+      <c r="O6" s="7">
         <v>0.89460154241645196</v>
       </c>
-      <c r="P6" s="6">
+      <c r="P6" s="5">
         <v>0.53</v>
       </c>
-      <c r="Q6" s="8">
+      <c r="Q6" s="7">
         <v>0.95471521942110105</v>
       </c>
-      <c r="R6" s="6">
+      <c r="R6" s="5">
         <v>0.71</v>
       </c>
-      <c r="T6" s="8">
+      <c r="T6" s="7">
         <v>0.84835900870729997</v>
       </c>
       <c r="V6" s="2">
@@ -818,11 +843,11 @@
     </row>
     <row r="7" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
-      <c r="K7" s="8"/>
-      <c r="M7" s="8"/>
-      <c r="O7" s="8"/>
-      <c r="Q7" s="8"/>
-      <c r="T7" s="8"/>
+      <c r="K7" s="7"/>
+      <c r="M7" s="7"/>
+      <c r="O7" s="7"/>
+      <c r="Q7" s="7"/>
+      <c r="T7" s="7"/>
       <c r="V7" s="2"/>
       <c r="W7" s="2"/>
       <c r="X7" s="2"/>
@@ -830,11 +855,11 @@
     </row>
     <row r="8" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A8" s="1"/>
-      <c r="K8" s="8"/>
-      <c r="M8" s="8"/>
-      <c r="O8" s="8"/>
-      <c r="Q8" s="8"/>
-      <c r="T8" s="8"/>
+      <c r="K8" s="7"/>
+      <c r="M8" s="7"/>
+      <c r="O8" s="7"/>
+      <c r="Q8" s="7"/>
+      <c r="T8" s="7"/>
       <c r="V8" s="2"/>
       <c r="W8" s="2"/>
       <c r="X8" s="2"/>
@@ -842,34 +867,48 @@
     </row>
     <row r="9" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A9" s="1"/>
-      <c r="K9" s="8"/>
-      <c r="M9" s="8"/>
-      <c r="O9" s="8"/>
-      <c r="Q9" s="8"/>
-      <c r="T9" s="8"/>
+      <c r="K9" s="7"/>
+      <c r="M9" s="7"/>
+      <c r="O9" s="7"/>
+      <c r="Q9" s="7"/>
+      <c r="T9" s="7"/>
       <c r="V9" s="2"/>
       <c r="W9" s="2"/>
       <c r="X9" s="2"/>
       <c r="Y9" s="2"/>
     </row>
     <row r="10" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A10" s="1"/>
-      <c r="K10" s="8"/>
-      <c r="M10" s="8"/>
-      <c r="O10" s="8"/>
-      <c r="Q10" s="8"/>
-      <c r="T10" s="8"/>
+      <c r="A10" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B10" t="s">
+        <v>25</v>
+      </c>
+      <c r="C10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D10" t="s">
+        <v>27</v>
+      </c>
+      <c r="E10">
+        <v>200</v>
+      </c>
+      <c r="K10" s="7"/>
+      <c r="M10" s="7"/>
+      <c r="O10" s="7"/>
+      <c r="Q10" s="7"/>
+      <c r="T10" s="7"/>
       <c r="V10" s="2"/>
       <c r="W10" s="2"/>
       <c r="X10" s="2"/>
       <c r="Y10" s="2"/>
     </row>
     <row r="11" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="K11" s="8"/>
-      <c r="M11" s="8"/>
-      <c r="O11" s="8"/>
-      <c r="Q11" s="8"/>
-      <c r="T11" s="8"/>
+      <c r="K11" s="7"/>
+      <c r="M11" s="7"/>
+      <c r="O11" s="7"/>
+      <c r="Q11" s="7"/>
+      <c r="T11" s="7"/>
       <c r="V11" s="2"/>
       <c r="W11" s="2"/>
       <c r="X11" s="2"/>
@@ -877,190 +916,190 @@
     </row>
     <row r="12" spans="1:25" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3"/>
-      <c r="K12" s="8"/>
-      <c r="L12" s="7"/>
-      <c r="M12" s="8"/>
-      <c r="N12" s="7"/>
-      <c r="O12" s="8"/>
-      <c r="P12" s="7"/>
-      <c r="Q12" s="8"/>
-      <c r="R12" s="7"/>
-      <c r="T12" s="8"/>
+      <c r="K12" s="7"/>
+      <c r="L12" s="6"/>
+      <c r="M12" s="7"/>
+      <c r="N12" s="6"/>
+      <c r="O12" s="7"/>
+      <c r="P12" s="6"/>
+      <c r="Q12" s="7"/>
+      <c r="R12" s="6"/>
+      <c r="T12" s="7"/>
       <c r="V12" s="2"/>
       <c r="W12" s="2"/>
       <c r="X12" s="2"/>
       <c r="Y12" s="2"/>
     </row>
     <row r="13" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="K13" s="8"/>
-      <c r="M13" s="8"/>
-      <c r="O13" s="8"/>
-      <c r="Q13" s="8"/>
-      <c r="T13" s="8"/>
+      <c r="K13" s="7"/>
+      <c r="M13" s="7"/>
+      <c r="O13" s="7"/>
+      <c r="Q13" s="7"/>
+      <c r="T13" s="7"/>
       <c r="V13" s="2"/>
       <c r="W13" s="2"/>
       <c r="X13" s="2"/>
       <c r="Y13" s="2"/>
     </row>
     <row r="14" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="K14" s="8"/>
-      <c r="M14" s="8"/>
-      <c r="O14" s="8"/>
-      <c r="Q14" s="8"/>
-      <c r="T14" s="8"/>
+      <c r="K14" s="7"/>
+      <c r="M14" s="7"/>
+      <c r="O14" s="7"/>
+      <c r="Q14" s="7"/>
+      <c r="T14" s="7"/>
       <c r="V14" s="2"/>
       <c r="W14" s="2"/>
       <c r="X14" s="2"/>
       <c r="Y14" s="2"/>
     </row>
     <row r="15" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="K15" s="8"/>
-      <c r="M15" s="8"/>
-      <c r="O15" s="8"/>
-      <c r="Q15" s="8"/>
-      <c r="T15" s="8"/>
+      <c r="K15" s="7"/>
+      <c r="M15" s="7"/>
+      <c r="O15" s="7"/>
+      <c r="Q15" s="7"/>
+      <c r="T15" s="7"/>
       <c r="V15" s="2"/>
       <c r="W15" s="2"/>
       <c r="X15" s="2"/>
       <c r="Y15" s="2"/>
     </row>
     <row r="16" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="K16" s="8"/>
-      <c r="M16" s="8"/>
-      <c r="O16" s="8"/>
-      <c r="Q16" s="8"/>
-      <c r="T16" s="8"/>
+      <c r="K16" s="7"/>
+      <c r="M16" s="7"/>
+      <c r="O16" s="7"/>
+      <c r="Q16" s="7"/>
+      <c r="T16" s="7"/>
       <c r="V16" s="2"/>
       <c r="W16" s="2"/>
       <c r="X16" s="2"/>
       <c r="Y16" s="2"/>
     </row>
     <row r="17" spans="11:25" x14ac:dyDescent="0.25">
-      <c r="K17" s="8"/>
-      <c r="M17" s="8"/>
-      <c r="O17" s="8"/>
-      <c r="Q17" s="8"/>
-      <c r="T17" s="8"/>
+      <c r="K17" s="7"/>
+      <c r="M17" s="7"/>
+      <c r="O17" s="7"/>
+      <c r="Q17" s="7"/>
+      <c r="T17" s="7"/>
       <c r="V17" s="2"/>
       <c r="W17" s="2"/>
       <c r="X17" s="2"/>
       <c r="Y17" s="2"/>
     </row>
     <row r="18" spans="11:25" x14ac:dyDescent="0.25">
-      <c r="K18" s="8"/>
-      <c r="M18" s="8"/>
-      <c r="O18" s="8"/>
-      <c r="Q18" s="8"/>
-      <c r="T18" s="8"/>
+      <c r="K18" s="7"/>
+      <c r="M18" s="7"/>
+      <c r="O18" s="7"/>
+      <c r="Q18" s="7"/>
+      <c r="T18" s="7"/>
       <c r="V18" s="2"/>
       <c r="W18" s="2"/>
       <c r="X18" s="2"/>
       <c r="Y18" s="2"/>
     </row>
     <row r="19" spans="11:25" x14ac:dyDescent="0.25">
-      <c r="K19" s="8"/>
-      <c r="M19" s="8"/>
-      <c r="O19" s="8"/>
-      <c r="Q19" s="8"/>
-      <c r="T19" s="8"/>
+      <c r="K19" s="7"/>
+      <c r="M19" s="7"/>
+      <c r="O19" s="7"/>
+      <c r="Q19" s="7"/>
+      <c r="T19" s="7"/>
       <c r="V19" s="2"/>
       <c r="W19" s="2"/>
       <c r="X19" s="2"/>
       <c r="Y19" s="2"/>
     </row>
     <row r="20" spans="11:25" x14ac:dyDescent="0.25">
-      <c r="K20" s="8"/>
-      <c r="M20" s="8"/>
-      <c r="O20" s="8"/>
-      <c r="Q20" s="8"/>
-      <c r="T20" s="8"/>
+      <c r="K20" s="7"/>
+      <c r="M20" s="7"/>
+      <c r="O20" s="7"/>
+      <c r="Q20" s="7"/>
+      <c r="T20" s="7"/>
       <c r="V20" s="2"/>
       <c r="W20" s="2"/>
       <c r="X20" s="2"/>
       <c r="Y20" s="2"/>
     </row>
     <row r="21" spans="11:25" x14ac:dyDescent="0.25">
-      <c r="K21" s="8"/>
-      <c r="M21" s="8"/>
-      <c r="O21" s="8"/>
-      <c r="Q21" s="8"/>
-      <c r="T21" s="8"/>
+      <c r="K21" s="7"/>
+      <c r="M21" s="7"/>
+      <c r="O21" s="7"/>
+      <c r="Q21" s="7"/>
+      <c r="T21" s="7"/>
       <c r="V21" s="2"/>
       <c r="W21" s="2"/>
       <c r="X21" s="2"/>
       <c r="Y21" s="2"/>
     </row>
     <row r="22" spans="11:25" x14ac:dyDescent="0.25">
-      <c r="K22" s="8"/>
-      <c r="M22" s="8"/>
-      <c r="O22" s="8"/>
-      <c r="Q22" s="8"/>
-      <c r="T22" s="8"/>
+      <c r="K22" s="7"/>
+      <c r="M22" s="7"/>
+      <c r="O22" s="7"/>
+      <c r="Q22" s="7"/>
+      <c r="T22" s="7"/>
       <c r="V22" s="2"/>
       <c r="W22" s="2"/>
       <c r="X22" s="2"/>
       <c r="Y22" s="2"/>
     </row>
     <row r="23" spans="11:25" x14ac:dyDescent="0.25">
-      <c r="K23" s="8"/>
-      <c r="M23" s="8"/>
-      <c r="O23" s="8"/>
-      <c r="Q23" s="8"/>
-      <c r="T23" s="8"/>
+      <c r="K23" s="7"/>
+      <c r="M23" s="7"/>
+      <c r="O23" s="7"/>
+      <c r="Q23" s="7"/>
+      <c r="T23" s="7"/>
       <c r="V23" s="2"/>
       <c r="W23" s="2"/>
       <c r="X23" s="2"/>
       <c r="Y23" s="2"/>
     </row>
     <row r="24" spans="11:25" x14ac:dyDescent="0.25">
-      <c r="K24" s="8"/>
-      <c r="M24" s="8"/>
-      <c r="O24" s="8"/>
-      <c r="Q24" s="8"/>
-      <c r="T24" s="8"/>
+      <c r="K24" s="7"/>
+      <c r="M24" s="7"/>
+      <c r="O24" s="7"/>
+      <c r="Q24" s="7"/>
+      <c r="T24" s="7"/>
       <c r="V24" s="2"/>
       <c r="W24" s="2"/>
       <c r="X24" s="2"/>
       <c r="Y24" s="2"/>
     </row>
     <row r="25" spans="11:25" x14ac:dyDescent="0.25">
-      <c r="K25" s="8"/>
-      <c r="M25" s="8"/>
-      <c r="O25" s="8"/>
-      <c r="Q25" s="8"/>
-      <c r="T25" s="8"/>
+      <c r="K25" s="7"/>
+      <c r="M25" s="7"/>
+      <c r="O25" s="7"/>
+      <c r="Q25" s="7"/>
+      <c r="T25" s="7"/>
       <c r="V25" s="2"/>
       <c r="W25" s="2"/>
       <c r="X25" s="2"/>
       <c r="Y25" s="2"/>
     </row>
     <row r="26" spans="11:25" x14ac:dyDescent="0.25">
-      <c r="O26" s="8"/>
-      <c r="Q26" s="8"/>
-      <c r="T26" s="8"/>
+      <c r="O26" s="7"/>
+      <c r="Q26" s="7"/>
+      <c r="T26" s="7"/>
       <c r="V26" s="2"/>
       <c r="W26" s="2"/>
       <c r="X26" s="2"/>
       <c r="Y26" s="2"/>
     </row>
     <row r="27" spans="11:25" x14ac:dyDescent="0.25">
-      <c r="O27" s="8"/>
-      <c r="Q27" s="8"/>
-      <c r="T27" s="8"/>
+      <c r="O27" s="7"/>
+      <c r="Q27" s="7"/>
+      <c r="T27" s="7"/>
       <c r="V27" s="2"/>
       <c r="W27" s="2"/>
       <c r="X27" s="2"/>
       <c r="Y27" s="2"/>
     </row>
     <row r="28" spans="11:25" x14ac:dyDescent="0.25">
-      <c r="Q28" s="8"/>
+      <c r="Q28" s="7"/>
       <c r="V28" s="2"/>
       <c r="W28" s="2"/>
       <c r="X28" s="2"/>
       <c r="Y28" s="2"/>
     </row>
     <row r="29" spans="11:25" x14ac:dyDescent="0.25">
-      <c r="Q29" s="8"/>
+      <c r="Q29" s="7"/>
       <c r="V29" s="2"/>
       <c r="W29" s="2"/>
       <c r="X29" s="2"/>

</xml_diff>